<commit_message>
fidelity_comparison: build disciplines from unified JSON pipeline
Construct F16Geom/F16Aero via f16a_spec_path and inject the L2 geom into aero L2/L3; regenerate the JSON/xlsx outputs.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/air_vehicle_design/sizing/examples/F16A/fidelity_comparison.xlsx
+++ b/air_vehicle_design/sizing/examples/F16A/fidelity_comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="756" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="756" uniqueCount="405">
   <si>
     <t>Row</t>
   </si>
@@ -592,130 +592,424 @@
     <t>0.0160</t>
   </si>
   <si>
+    <t>0.0222</t>
+  </si>
+  <si>
+    <t>0.0280</t>
+  </si>
+  <si>
+    <t>0.1800</t>
+  </si>
+  <si>
+    <t>0.1903</t>
+  </si>
+  <si>
+    <t>0.2700</t>
+  </si>
+  <si>
+    <t>0.3600</t>
+  </si>
+  <si>
+    <t>0.9000</t>
+  </si>
+  <si>
+    <t>-0.0500</t>
+  </si>
+  <si>
+    <t>-0.1000</t>
+  </si>
+  <si>
+    <t>0.0350</t>
+  </si>
+  <si>
+    <t>0.0850</t>
+  </si>
+  <si>
+    <t>0.0510</t>
+  </si>
+  <si>
+    <t>0.1010</t>
+  </si>
+  <si>
+    <t>0.2000</t>
+  </si>
+  <si>
+    <t>0.6000</t>
+  </si>
+  <si>
+    <t>1.1000</t>
+  </si>
+  <si>
+    <t>1.5000</t>
+  </si>
+  <si>
+    <t>0.2880</t>
+  </si>
+  <si>
+    <t>0.2467</t>
+  </si>
+  <si>
+    <t>0.4837</t>
+  </si>
+  <si>
+    <t>0.6854</t>
+  </si>
+  <si>
+    <t>0.3232</t>
+  </si>
+  <si>
+    <t>0.8337</t>
+  </si>
+  <si>
+    <t>0.800</t>
+  </si>
+  <si>
+    <t>L1_err</t>
+  </si>
+  <si>
+    <t>-0.2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - </t>
+  </si>
+  <si>
+    <t>+28.6%</t>
+  </si>
+  <si>
+    <t>+11.0%</t>
+  </si>
+  <si>
+    <t>-5.9%</t>
+  </si>
+  <si>
+    <t>-51.4%</t>
+  </si>
+  <si>
+    <t>-29.9%</t>
+  </si>
+  <si>
+    <t>-25.0%</t>
+  </si>
+  <si>
+    <t>+55.2%</t>
+  </si>
+  <si>
+    <t>+49.0%</t>
+  </si>
+  <si>
+    <t>+7.3%</t>
+  </si>
+  <si>
+    <t>-1.9%</t>
+  </si>
+  <si>
+    <t>-8.8%</t>
+  </si>
+  <si>
+    <t>+62.9%</t>
+  </si>
+  <si>
+    <t>-31.4%</t>
+  </si>
+  <si>
+    <t>+35.8%</t>
+  </si>
+  <si>
+    <t>-14.0%</t>
+  </si>
+  <si>
+    <t>+5.0%</t>
+  </si>
+  <si>
+    <t>-39.3%</t>
+  </si>
+  <si>
+    <t>-15.3%</t>
+  </si>
+  <si>
+    <t>+55.1%</t>
+  </si>
+  <si>
+    <t>-100.0%</t>
+  </si>
+  <si>
+    <t>-28.8%</t>
+  </si>
+  <si>
+    <t>+130.2%</t>
+  </si>
+  <si>
+    <t>-31.1%</t>
+  </si>
+  <si>
+    <t>+96.3%</t>
+  </si>
+  <si>
+    <t>+45.4%</t>
+  </si>
+  <si>
+    <t>+0.5%</t>
+  </si>
+  <si>
+    <t>-16.2%</t>
+  </si>
+  <si>
+    <t>+89.8%</t>
+  </si>
+  <si>
+    <t>-13.1%</t>
+  </si>
+  <si>
+    <t>-2.3%</t>
+  </si>
+  <si>
+    <t>+0.0%</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>16091</t>
+  </si>
+  <si>
+    <t>0.5128</t>
+  </si>
+  <si>
+    <t>1766</t>
+  </si>
+  <si>
+    <t>217</t>
+  </si>
+  <si>
+    <t>3600</t>
+  </si>
+  <si>
+    <t>1035</t>
+  </si>
+  <si>
+    <t>3939</t>
+  </si>
+  <si>
+    <t>5334</t>
+  </si>
+  <si>
+    <t>1466.8</t>
+  </si>
+  <si>
+    <t>46.50</t>
+  </si>
+  <si>
+    <t>396.4</t>
+  </si>
+  <si>
+    <t>101.4</t>
+  </si>
+  <si>
+    <t>83.1</t>
+  </si>
+  <si>
+    <t>730.3</t>
+  </si>
+  <si>
+    <t>155.6</t>
+  </si>
+  <si>
+    <t>0.0171</t>
+  </si>
+  <si>
+    <t>0.0080</t>
+  </si>
+  <si>
+    <t>0.0070</t>
+  </si>
+  <si>
+    <t>0.0060</t>
+  </si>
+  <si>
     <t>0.1168</t>
   </si>
   <si>
     <t>0.9086</t>
   </si>
   <si>
-    <t>0.9000</t>
-  </si>
-  <si>
-    <t>-0.0500</t>
-  </si>
-  <si>
-    <t>-0.1000</t>
-  </si>
-  <si>
-    <t>0.0350</t>
-  </si>
-  <si>
-    <t>0.0850</t>
-  </si>
-  <si>
-    <t>0.0510</t>
-  </si>
-  <si>
-    <t>0.1010</t>
-  </si>
-  <si>
-    <t>0.2000</t>
-  </si>
-  <si>
-    <t>0.6000</t>
-  </si>
-  <si>
-    <t>1.1000</t>
-  </si>
-  <si>
-    <t>1.5000</t>
+    <t>0.9141</t>
+  </si>
+  <si>
+    <t>3.0365</t>
+  </si>
+  <si>
+    <t>2.9179</t>
+  </si>
+  <si>
+    <t>0.0344</t>
+  </si>
+  <si>
+    <t>0.0488</t>
+  </si>
+  <si>
+    <t>0.0515</t>
+  </si>
+  <si>
+    <t>0.0659</t>
+  </si>
+  <si>
+    <t>0.3291</t>
+  </si>
+  <si>
+    <t>0.4387</t>
+  </si>
+  <si>
+    <t>1.2431</t>
+  </si>
+  <si>
+    <t>1.3528</t>
+  </si>
+  <si>
+    <t>0.0257</t>
+  </si>
+  <si>
+    <t>0.0456</t>
+  </si>
+  <si>
+    <t>0.0079</t>
   </si>
   <si>
     <t>0.2760</t>
   </si>
   <si>
-    <t>-0.0000</t>
+    <t>-0.0052</t>
+  </si>
+  <si>
+    <t>0.0084</t>
   </si>
   <si>
     <t>0.2261</t>
   </si>
   <si>
-    <t>0.4837</t>
-  </si>
-  <si>
-    <t>0.6854</t>
-  </si>
-  <si>
-    <t>0.3232</t>
-  </si>
-  <si>
-    <t>0.8337</t>
-  </si>
-  <si>
-    <t>0.800</t>
-  </si>
-  <si>
-    <t>L1_err</t>
-  </si>
-  <si>
-    <t>-0.2%</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> - </t>
-  </si>
-  <si>
-    <t>+28.6%</t>
-  </si>
-  <si>
-    <t>+11.0%</t>
-  </si>
-  <si>
-    <t>-5.9%</t>
-  </si>
-  <si>
-    <t>-65.0%</t>
-  </si>
-  <si>
-    <t>-60.0%</t>
-  </si>
-  <si>
-    <t>-57.1%</t>
+    <t>0.3674</t>
+  </si>
+  <si>
+    <t>0.2204</t>
+  </si>
+  <si>
+    <t>0.7526</t>
+  </si>
+  <si>
+    <t>0.4516</t>
+  </si>
+  <si>
+    <t>0.5494</t>
+  </si>
+  <si>
+    <t>0.3089</t>
+  </si>
+  <si>
+    <t>0.1875</t>
+  </si>
+  <si>
+    <t>0.1125</t>
+  </si>
+  <si>
+    <t>0.6007</t>
+  </si>
+  <si>
+    <t>0.3546</t>
+  </si>
+  <si>
+    <t>0.8608</t>
+  </si>
+  <si>
+    <t>0.5028</t>
+  </si>
+  <si>
+    <t>0.903</t>
+  </si>
+  <si>
+    <t>1.007</t>
+  </si>
+  <si>
+    <t>L2_err</t>
+  </si>
+  <si>
+    <t>-16.0%</t>
+  </si>
+  <si>
+    <t>-4.6%</t>
+  </si>
+  <si>
+    <t>-11.7%</t>
+  </si>
+  <si>
+    <t>+2.7%</t>
+  </si>
+  <si>
+    <t>-2.9%</t>
+  </si>
+  <si>
+    <t>-30.2%</t>
+  </si>
+  <si>
+    <t>-21.8%</t>
+  </si>
+  <si>
+    <t>+7.0%</t>
+  </si>
+  <si>
+    <t>-2.1%</t>
+  </si>
+  <si>
+    <t>+1.1%</t>
+  </si>
+  <si>
+    <t>+1.8%</t>
+  </si>
+  <si>
+    <t>+8.0%</t>
+  </si>
+  <si>
+    <t>+274.7%</t>
   </si>
   <si>
     <t>+0.7%</t>
   </si>
   <si>
+    <t>-82.5%</t>
+  </si>
+  <si>
+    <t>-83.9%</t>
+  </si>
+  <si>
     <t>-0.0%</t>
   </si>
   <si>
-    <t>+0.0%</t>
-  </si>
-  <si>
     <t>-0.7%</t>
   </si>
   <si>
-    <t>-8.8%</t>
-  </si>
-  <si>
-    <t>-1.9%</t>
-  </si>
-  <si>
-    <t>+62.9%</t>
-  </si>
-  <si>
-    <t>-31.4%</t>
-  </si>
-  <si>
-    <t>+35.8%</t>
-  </si>
-  <si>
-    <t>-14.0%</t>
-  </si>
-  <si>
-    <t>+5.0%</t>
-  </si>
-  <si>
-    <t>-65.3%</t>
+    <t>-7.4%</t>
+  </si>
+  <si>
+    <t>-2.4%</t>
+  </si>
+  <si>
+    <t>-6.2%</t>
+  </si>
+  <si>
+    <t>-0.9%</t>
+  </si>
+  <si>
+    <t>+6.3%</t>
+  </si>
+  <si>
+    <t>+12.8%</t>
+  </si>
+  <si>
+    <t>-2.8%</t>
+  </si>
+  <si>
+    <t>-5.3%</t>
+  </si>
+  <si>
+    <t>-82.9%</t>
   </si>
   <si>
     <t>-18.8%</t>
@@ -724,267 +1018,48 @@
     <t>+0.6%</t>
   </si>
   <si>
-    <t>-100.0%</t>
-  </si>
-  <si>
-    <t>-59.3%</t>
+    <t>-21.2%</t>
+  </si>
+  <si>
+    <t>-80.0%</t>
   </si>
   <si>
     <t>+120.6%</t>
   </si>
   <si>
-    <t>-60.6%</t>
+    <t>-79.4%</t>
   </si>
   <si>
     <t>+80.0%</t>
   </si>
   <si>
-    <t>+45.4%</t>
-  </si>
-  <si>
-    <t>+0.5%</t>
-  </si>
-  <si>
-    <t>-16.2%</t>
-  </si>
-  <si>
-    <t>+89.8%</t>
-  </si>
-  <si>
-    <t>-13.1%</t>
-  </si>
-  <si>
-    <t>-2.3%</t>
-  </si>
-  <si>
-    <t>L2</t>
-  </si>
-  <si>
-    <t>16091</t>
-  </si>
-  <si>
-    <t>0.5128</t>
-  </si>
-  <si>
-    <t>1766</t>
-  </si>
-  <si>
-    <t>217</t>
-  </si>
-  <si>
-    <t>3600</t>
-  </si>
-  <si>
-    <t>1035</t>
-  </si>
-  <si>
-    <t>3939</t>
-  </si>
-  <si>
-    <t>5334</t>
-  </si>
-  <si>
-    <t>1466.8</t>
-  </si>
-  <si>
-    <t>46.50</t>
-  </si>
-  <si>
-    <t>396.4</t>
-  </si>
-  <si>
-    <t>101.4</t>
-  </si>
-  <si>
-    <t>83.1</t>
-  </si>
-  <si>
-    <t>730.3</t>
-  </si>
-  <si>
-    <t>155.6</t>
-  </si>
-  <si>
-    <t>0.8625</t>
-  </si>
-  <si>
-    <t>2.9310</t>
-  </si>
-  <si>
-    <t>3.1387</t>
-  </si>
-  <si>
-    <t>0.0344</t>
-  </si>
-  <si>
-    <t>0.0488</t>
-  </si>
-  <si>
-    <t>0.0504</t>
-  </si>
-  <si>
-    <t>0.0648</t>
-  </si>
-  <si>
-    <t>0.3105</t>
-  </si>
-  <si>
-    <t>0.4140</t>
-  </si>
-  <si>
-    <t>1.1730</t>
-  </si>
-  <si>
-    <t>1.2765</t>
-  </si>
-  <si>
-    <t>0.0216</t>
-  </si>
-  <si>
-    <t>0.0383</t>
-  </si>
-  <si>
-    <t>-0.0073</t>
-  </si>
-  <si>
-    <t>0.3674</t>
-  </si>
-  <si>
-    <t>0.2204</t>
-  </si>
-  <si>
-    <t>0.7526</t>
-  </si>
-  <si>
-    <t>0.4516</t>
-  </si>
-  <si>
-    <t>0.5494</t>
-  </si>
-  <si>
-    <t>0.3089</t>
-  </si>
-  <si>
-    <t>0.1875</t>
-  </si>
-  <si>
-    <t>0.1125</t>
-  </si>
-  <si>
-    <t>0.6007</t>
-  </si>
-  <si>
-    <t>0.3546</t>
-  </si>
-  <si>
-    <t>0.8608</t>
-  </si>
-  <si>
-    <t>0.5028</t>
-  </si>
-  <si>
-    <t>0.903</t>
-  </si>
-  <si>
-    <t>1.007</t>
-  </si>
-  <si>
-    <t>L2_err</t>
-  </si>
-  <si>
-    <t>-16.0%</t>
-  </si>
-  <si>
-    <t>-4.6%</t>
-  </si>
-  <si>
-    <t>-11.7%</t>
-  </si>
-  <si>
-    <t>+2.7%</t>
-  </si>
-  <si>
-    <t>-2.9%</t>
-  </si>
-  <si>
-    <t>-30.2%</t>
-  </si>
-  <si>
-    <t>-21.8%</t>
-  </si>
-  <si>
-    <t>+7.0%</t>
-  </si>
-  <si>
-    <t>-2.1%</t>
-  </si>
-  <si>
-    <t>+1.1%</t>
-  </si>
-  <si>
-    <t>+1.8%</t>
-  </si>
-  <si>
-    <t>+8.0%</t>
-  </si>
-  <si>
-    <t>+274.7%</t>
-  </si>
-  <si>
-    <t>-12.6%</t>
-  </si>
-  <si>
-    <t>-5.8%</t>
+    <t>+10.4%</t>
+  </si>
+  <si>
+    <t>+28.8%</t>
+  </si>
+  <si>
+    <t>-4.8%</t>
+  </si>
+  <si>
+    <t>+64.1%</t>
+  </si>
+  <si>
+    <t>+10.1%</t>
+  </si>
+  <si>
+    <t>+28.4%</t>
+  </si>
+  <si>
+    <t>+7.9%</t>
+  </si>
+  <si>
+    <t>+57.0%</t>
   </si>
   <si>
     <t>+0.9%</t>
   </si>
   <si>
-    <t>-3.1%</t>
-  </si>
-  <si>
-    <t>+4.5%</t>
-  </si>
-  <si>
-    <t>+6.5%</t>
-  </si>
-  <si>
-    <t>-6.3%</t>
-  </si>
-  <si>
-    <t>-8.2%</t>
-  </si>
-  <si>
-    <t>-10.7%</t>
-  </si>
-  <si>
-    <t>+11.3%</t>
-  </si>
-  <si>
-    <t>+10.4%</t>
-  </si>
-  <si>
-    <t>+28.8%</t>
-  </si>
-  <si>
-    <t>-4.8%</t>
-  </si>
-  <si>
-    <t>+64.1%</t>
-  </si>
-  <si>
-    <t>+10.1%</t>
-  </si>
-  <si>
-    <t>+28.4%</t>
-  </si>
-  <si>
-    <t>+7.9%</t>
-  </si>
-  <si>
-    <t>+57.0%</t>
-  </si>
-  <si>
     <t>+13.4%</t>
   </si>
   <si>
@@ -1021,19 +1096,22 @@
     <t>4541</t>
   </si>
   <si>
-    <t>0.0159</t>
-  </si>
-  <si>
-    <t>0.0142</t>
-  </si>
-  <si>
-    <t>0.0137</t>
-  </si>
-  <si>
-    <t>0.0286</t>
-  </si>
-  <si>
-    <t>0.0261</t>
+    <t>0.0148</t>
+  </si>
+  <si>
+    <t>0.0143</t>
+  </si>
+  <si>
+    <t>0.0459</t>
+  </si>
+  <si>
+    <t>0.0421</t>
+  </si>
+  <si>
+    <t>3.0240</t>
+  </si>
+  <si>
+    <t>3.2579</t>
   </si>
   <si>
     <t>0.0342</t>
@@ -1042,43 +1120,40 @@
     <t>0.0486</t>
   </si>
   <si>
-    <t>0.0494</t>
-  </si>
-  <si>
-    <t>0.0638</t>
-  </si>
-  <si>
-    <t>0.3351</t>
-  </si>
-  <si>
-    <t>0.4469</t>
-  </si>
-  <si>
-    <t>1.2351</t>
-  </si>
-  <si>
-    <t>1.3469</t>
-  </si>
-  <si>
-    <t>0.0385</t>
-  </si>
-  <si>
-    <t>0.0291</t>
-  </si>
-  <si>
-    <t>0.0154</t>
-  </si>
-  <si>
-    <t>-0.0071</t>
-  </si>
-  <si>
-    <t>0.0143</t>
-  </si>
-  <si>
-    <t>0.0168</t>
-  </si>
-  <si>
-    <t>0.0303</t>
+    <t>0.0503</t>
+  </si>
+  <si>
+    <t>0.0647</t>
+  </si>
+  <si>
+    <t>0.3537</t>
+  </si>
+  <si>
+    <t>0.4716</t>
+  </si>
+  <si>
+    <t>1.2677</t>
+  </si>
+  <si>
+    <t>1.3856</t>
+  </si>
+  <si>
+    <t>0.0462</t>
+  </si>
+  <si>
+    <t>0.0161</t>
+  </si>
+  <si>
+    <t>-0.0074</t>
+  </si>
+  <si>
+    <t>0.0150</t>
+  </si>
+  <si>
+    <t>0.0176</t>
+  </si>
+  <si>
+    <t>0.0481</t>
   </si>
   <si>
     <t>L3_err</t>
@@ -1099,61 +1174,61 @@
     <t>+4.8%</t>
   </si>
   <si>
-    <t>-0.9%</t>
-  </si>
-  <si>
     <t>-35.5%</t>
   </si>
   <si>
     <t>-33.4%</t>
   </si>
   <si>
-    <t>-16.6%</t>
-  </si>
-  <si>
-    <t>-70.1%</t>
-  </si>
-  <si>
-    <t>-28.4%</t>
-  </si>
-  <si>
-    <t>-30.0%</t>
-  </si>
-  <si>
-    <t>-5.0%</t>
-  </si>
-  <si>
-    <t>+2.9%</t>
-  </si>
-  <si>
-    <t>+14.9%</t>
-  </si>
-  <si>
-    <t>-3.4%</t>
-  </si>
-  <si>
-    <t>-5.7%</t>
-  </si>
-  <si>
-    <t>-36.8%</t>
-  </si>
-  <si>
-    <t>-9.7%</t>
-  </si>
-  <si>
-    <t>+7.3%</t>
-  </si>
-  <si>
-    <t>-15.7%</t>
-  </si>
-  <si>
-    <t>-25.9%</t>
-  </si>
-  <si>
-    <t>-1.2%</t>
-  </si>
-  <si>
-    <t>-25.4%</t>
+    <t>+0.3%</t>
+  </si>
+  <si>
+    <t>-12.7%</t>
+  </si>
+  <si>
+    <t>-68.7%</t>
+  </si>
+  <si>
+    <t>+15.0%</t>
+  </si>
+  <si>
+    <t>+12.9%</t>
+  </si>
+  <si>
+    <t>+4.7%</t>
+  </si>
+  <si>
+    <t>-3.2%</t>
+  </si>
+  <si>
+    <t>+4.4%</t>
+  </si>
+  <si>
+    <t>+21.3%</t>
+  </si>
+  <si>
+    <t>+6.7%</t>
+  </si>
+  <si>
+    <t>-0.8%</t>
+  </si>
+  <si>
+    <t>-3.0%</t>
+  </si>
+  <si>
+    <t>+12.6%</t>
+  </si>
+  <si>
+    <t>-11.6%</t>
+  </si>
+  <si>
+    <t>+17.6%</t>
+  </si>
+  <si>
+    <t>+3.6%</t>
+  </si>
+  <si>
+    <t>+18.4%</t>
   </si>
 </sst>
 </file>
@@ -1227,19 +1302,19 @@
         <v>186</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>325</v>
+        <v>350</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>355</v>
+        <v>380</v>
       </c>
     </row>
     <row r="2">
@@ -1285,19 +1360,19 @@
         <v>187</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>326</v>
+        <v>351</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>356</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4">
@@ -1314,19 +1389,19 @@
         <v>188</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>327</v>
+        <v>352</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>356</v>
+        <v>381</v>
       </c>
     </row>
     <row r="5">
@@ -1343,19 +1418,19 @@
         <v>113</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>328</v>
+        <v>353</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6">
@@ -1372,19 +1447,19 @@
         <v>113</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F6" s="0" t="s">
         <v>89</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>224</v>
+        <v>249</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>329</v>
+        <v>354</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>358</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7">
@@ -1401,19 +1476,19 @@
         <v>113</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>330</v>
+        <v>355</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>359</v>
+        <v>384</v>
       </c>
     </row>
     <row r="8">
@@ -1430,19 +1505,19 @@
         <v>113</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>331</v>
+        <v>356</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>360</v>
+        <v>385</v>
       </c>
     </row>
     <row r="9">
@@ -1459,19 +1534,19 @@
         <v>113</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>332</v>
+        <v>357</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>361</v>
+        <v>326</v>
       </c>
     </row>
     <row r="10">
@@ -1488,19 +1563,19 @@
         <v>113</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>333</v>
+        <v>358</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>362</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11">
@@ -1517,19 +1592,19 @@
         <v>113</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>334</v>
+        <v>359</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>363</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12">
@@ -1575,19 +1650,19 @@
         <v>189</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
       <c r="H13" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="14">
@@ -1604,19 +1679,19 @@
         <v>190</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="H14" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="15">
@@ -1633,19 +1708,19 @@
         <v>113</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="H15" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16">
@@ -1662,19 +1737,19 @@
         <v>113</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="H16" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="17">
@@ -1691,19 +1766,19 @@
         <v>113</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="H17" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="18">
@@ -1720,19 +1795,19 @@
         <v>113</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="H18" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="19">
@@ -1749,19 +1824,19 @@
         <v>113</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="H19" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I19" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20">
@@ -1807,19 +1882,19 @@
         <v>191</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>191</v>
+        <v>266</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>218</v>
+        <v>318</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>335</v>
+        <v>102</v>
       </c>
       <c r="I21" s="0" t="s">
-        <v>311</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22">
@@ -1836,19 +1911,19 @@
         <v>191</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>191</v>
+        <v>266</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>218</v>
+        <v>318</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>336</v>
+        <v>360</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>364</v>
+        <v>389</v>
       </c>
     </row>
     <row r="23">
@@ -1862,22 +1937,22 @@
         <v>158</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>191</v>
+        <v>267</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>219</v>
+        <v>319</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>337</v>
+        <v>361</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>365</v>
+        <v>390</v>
       </c>
     </row>
     <row r="24">
@@ -1891,22 +1966,22 @@
         <v>158</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>191</v>
+        <v>268</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>220</v>
+        <v>319</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>338</v>
+        <v>362</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>366</v>
+        <v>391</v>
       </c>
     </row>
     <row r="25">
@@ -1920,22 +1995,22 @@
         <v>158</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>191</v>
+        <v>269</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>221</v>
+        <v>320</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>339</v>
+        <v>363</v>
       </c>
       <c r="I25" s="0" t="s">
-        <v>367</v>
+        <v>392</v>
       </c>
     </row>
     <row r="26">
@@ -1949,22 +2024,22 @@
         <v>158</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>222</v>
+        <v>318</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="I26" s="0" t="s">
-        <v>222</v>
+        <v>318</v>
       </c>
     </row>
     <row r="27">
@@ -1978,22 +2053,22 @@
         <v>158</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>222</v>
+        <v>318</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="I27" s="0" t="s">
-        <v>222</v>
+        <v>318</v>
       </c>
     </row>
     <row r="28">
@@ -2007,22 +2082,22 @@
         <v>158</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>107</v>
+        <v>195</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F28" s="0" t="s">
         <v>107</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>223</v>
+        <v>321</v>
       </c>
       <c r="H28" s="0" t="s">
         <v>107</v>
       </c>
       <c r="I28" s="0" t="s">
-        <v>223</v>
+        <v>321</v>
       </c>
     </row>
     <row r="29">
@@ -2036,22 +2111,22 @@
         <v>158</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>108</v>
+        <v>196</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F29" s="0" t="s">
         <v>108</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>224</v>
+        <v>249</v>
       </c>
       <c r="H29" s="0" t="s">
         <v>108</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>224</v>
+        <v>249</v>
       </c>
     </row>
     <row r="30">
@@ -2065,22 +2140,22 @@
         <v>158</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>109</v>
+        <v>197</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="F30" s="0" t="s">
         <v>109</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>224</v>
+        <v>249</v>
       </c>
       <c r="H30" s="0" t="s">
         <v>109</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>224</v>
+        <v>249</v>
       </c>
     </row>
     <row r="31">
@@ -2094,22 +2169,22 @@
         <v>159</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>193</v>
+        <v>113</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>193</v>
+        <v>271</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>225</v>
+        <v>322</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>193</v>
+        <v>271</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>225</v>
+        <v>322</v>
       </c>
     </row>
     <row r="32">
@@ -2123,22 +2198,22 @@
         <v>160</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="G32" s="0" t="s">
-        <v>305</v>
+        <v>323</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>194</v>
+        <v>272</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>226</v>
+        <v>323</v>
       </c>
     </row>
     <row r="33">
@@ -2155,19 +2230,19 @@
         <v>113</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>306</v>
+        <v>324</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>264</v>
+        <v>364</v>
       </c>
       <c r="I33" s="0" t="s">
-        <v>306</v>
+        <v>329</v>
       </c>
     </row>
     <row r="34">
@@ -2184,19 +2259,19 @@
         <v>113</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>307</v>
+        <v>325</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>265</v>
+        <v>365</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>307</v>
+        <v>393</v>
       </c>
     </row>
     <row r="35">
@@ -2239,22 +2314,22 @@
         <v>162</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="I36" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="37">
@@ -2268,22 +2343,22 @@
         <v>162</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="38">
@@ -2297,22 +2372,22 @@
         <v>163</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H38" s="0" t="s">
-        <v>340</v>
+        <v>366</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="39">
@@ -2326,22 +2401,22 @@
         <v>163</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H39" s="0" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="I39" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="40">
@@ -2355,22 +2430,22 @@
         <v>164</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>368</v>
+        <v>394</v>
       </c>
     </row>
     <row r="41">
@@ -2384,22 +2459,22 @@
         <v>165</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>309</v>
+        <v>327</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>343</v>
+        <v>369</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>369</v>
+        <v>395</v>
       </c>
     </row>
     <row r="42">
@@ -2413,22 +2488,22 @@
         <v>166</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="H42" s="0" t="s">
-        <v>344</v>
+        <v>370</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>370</v>
+        <v>396</v>
       </c>
     </row>
     <row r="43">
@@ -2442,22 +2517,22 @@
         <v>167</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>311</v>
+        <v>322</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>345</v>
+        <v>371</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>301</v>
+        <v>397</v>
       </c>
     </row>
     <row r="44">
@@ -2471,22 +2546,22 @@
         <v>168</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>312</v>
+        <v>329</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>371</v>
+        <v>398</v>
       </c>
     </row>
     <row r="45">
@@ -2500,22 +2575,22 @@
         <v>169</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>313</v>
+        <v>330</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>347</v>
+        <v>373</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>372</v>
+        <v>399</v>
       </c>
     </row>
     <row r="46">
@@ -2532,19 +2607,19 @@
         <v>113</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H46" s="0" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="I46" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="47">
@@ -2561,19 +2636,19 @@
         <v>113</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F47" s="0" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>348</v>
+        <v>103</v>
       </c>
       <c r="I47" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="48">
@@ -2616,22 +2691,22 @@
         <v>170</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F49" s="0" t="s">
-        <v>191</v>
+        <v>285</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>233</v>
+        <v>331</v>
       </c>
       <c r="H49" s="0" t="s">
-        <v>349</v>
+        <v>374</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
     </row>
     <row r="50">
@@ -2645,22 +2720,22 @@
         <v>170</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>205</v>
+        <v>286</v>
       </c>
       <c r="G50" s="0" t="s">
-        <v>234</v>
+        <v>332</v>
       </c>
       <c r="H50" s="0" t="s">
-        <v>205</v>
+        <v>286</v>
       </c>
       <c r="I50" s="0" t="s">
-        <v>234</v>
+        <v>332</v>
       </c>
     </row>
     <row r="51">
@@ -2706,19 +2781,19 @@
         <v>191</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F52" s="0" t="s">
-        <v>191</v>
+        <v>266</v>
       </c>
       <c r="G52" s="0" t="s">
-        <v>218</v>
+        <v>318</v>
       </c>
       <c r="H52" s="0" t="s">
-        <v>350</v>
+        <v>375</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>374</v>
+        <v>330</v>
       </c>
     </row>
     <row r="53">
@@ -2732,22 +2807,22 @@
         <v>171</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F53" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>235</v>
+        <v>333</v>
       </c>
       <c r="H53" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>235</v>
+        <v>333</v>
       </c>
     </row>
     <row r="54">
@@ -2761,22 +2836,22 @@
         <v>171</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>206</v>
+        <v>125</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F54" s="0" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>314</v>
+        <v>334</v>
       </c>
       <c r="H54" s="0" t="s">
-        <v>351</v>
+        <v>376</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>375</v>
+        <v>400</v>
       </c>
     </row>
     <row r="55">
@@ -2793,19 +2868,19 @@
         <v>191</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F55" s="0" t="s">
-        <v>191</v>
+        <v>266</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>218</v>
+        <v>318</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>352</v>
+        <v>377</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>376</v>
+        <v>401</v>
       </c>
     </row>
     <row r="56">
@@ -2819,22 +2894,22 @@
         <v>171</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>235</v>
+        <v>333</v>
       </c>
       <c r="H56" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>235</v>
+        <v>333</v>
       </c>
     </row>
     <row r="57">
@@ -2848,22 +2923,22 @@
         <v>171</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>206</v>
+        <v>125</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>314</v>
+        <v>334</v>
       </c>
       <c r="H57" s="0" t="s">
-        <v>351</v>
+        <v>376</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>375</v>
+        <v>400</v>
       </c>
     </row>
     <row r="58">
@@ -2877,22 +2952,22 @@
         <v>171</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>191</v>
+        <v>285</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>237</v>
+        <v>335</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>349</v>
+        <v>374</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>377</v>
+        <v>402</v>
       </c>
     </row>
     <row r="59">
@@ -2906,22 +2981,22 @@
         <v>171</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>205</v>
+        <v>286</v>
       </c>
       <c r="G59" s="0" t="s">
-        <v>238</v>
+        <v>336</v>
       </c>
       <c r="H59" s="0" t="s">
-        <v>205</v>
+        <v>286</v>
       </c>
       <c r="I59" s="0" t="s">
-        <v>238</v>
+        <v>336</v>
       </c>
     </row>
     <row r="60">
@@ -2938,19 +3013,19 @@
         <v>125</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F60" s="0" t="s">
         <v>125</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H60" s="0" t="s">
         <v>125</v>
       </c>
       <c r="I60" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="61">
@@ -2967,19 +3042,19 @@
         <v>191</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>191</v>
+        <v>266</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>218</v>
+        <v>318</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>353</v>
+        <v>378</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>378</v>
+        <v>403</v>
       </c>
     </row>
     <row r="62">
@@ -2993,22 +3068,22 @@
         <v>171</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="G62" s="0" t="s">
-        <v>235</v>
+        <v>333</v>
       </c>
       <c r="H62" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="I62" s="0" t="s">
-        <v>235</v>
+        <v>333</v>
       </c>
     </row>
     <row r="63">
@@ -3022,22 +3097,22 @@
         <v>171</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>206</v>
+        <v>125</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="G63" s="0" t="s">
-        <v>314</v>
+        <v>334</v>
       </c>
       <c r="H63" s="0" t="s">
-        <v>351</v>
+        <v>376</v>
       </c>
       <c r="I63" s="0" t="s">
-        <v>375</v>
+        <v>400</v>
       </c>
     </row>
     <row r="64">
@@ -3051,22 +3126,22 @@
         <v>171</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>191</v>
+        <v>288</v>
       </c>
       <c r="G64" s="0" t="s">
-        <v>239</v>
+        <v>337</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>354</v>
+        <v>379</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>379</v>
+        <v>404</v>
       </c>
     </row>
     <row r="65">
@@ -3080,22 +3155,22 @@
         <v>171</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>207</v>
+        <v>289</v>
       </c>
       <c r="G65" s="0" t="s">
-        <v>240</v>
+        <v>338</v>
       </c>
       <c r="H65" s="0" t="s">
-        <v>207</v>
+        <v>289</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>240</v>
+        <v>338</v>
       </c>
     </row>
     <row r="66">
@@ -3112,19 +3187,19 @@
         <v>125</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F66" s="0" t="s">
         <v>125</v>
       </c>
       <c r="G66" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="H66" s="0" t="s">
         <v>125</v>
       </c>
       <c r="I66" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="67">
@@ -3141,19 +3216,19 @@
         <v>191</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>191</v>
+        <v>266</v>
       </c>
       <c r="G67" s="0" t="s">
-        <v>218</v>
+        <v>318</v>
       </c>
       <c r="H67" s="0" t="s">
-        <v>336</v>
+        <v>360</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>364</v>
+        <v>389</v>
       </c>
     </row>
     <row r="68">
@@ -3167,22 +3242,22 @@
         <v>171</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F68" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="G68" s="0" t="s">
-        <v>235</v>
+        <v>333</v>
       </c>
       <c r="H68" s="0" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>235</v>
+        <v>333</v>
       </c>
     </row>
     <row r="69">
@@ -3196,22 +3271,22 @@
         <v>171</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>206</v>
+        <v>125</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F69" s="0" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="G69" s="0" t="s">
-        <v>314</v>
+        <v>334</v>
       </c>
       <c r="H69" s="0" t="s">
-        <v>351</v>
+        <v>376</v>
       </c>
       <c r="I69" s="0" t="s">
-        <v>375</v>
+        <v>400</v>
       </c>
     </row>
     <row r="70">
@@ -3254,22 +3329,22 @@
         <v>172</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E71" s="0" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="G71" s="0" t="s">
-        <v>315</v>
+        <v>339</v>
       </c>
       <c r="H71" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I71" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="72">
@@ -3286,19 +3361,19 @@
         <v>113</v>
       </c>
       <c r="E72" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="G72" s="0" t="s">
-        <v>316</v>
+        <v>340</v>
       </c>
       <c r="H72" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I72" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="73">
@@ -3312,22 +3387,22 @@
         <v>174</v>
       </c>
       <c r="D73" s="0" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E73" s="0" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="G73" s="0" t="s">
-        <v>315</v>
+        <v>339</v>
       </c>
       <c r="H73" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="74">
@@ -3344,19 +3419,19 @@
         <v>113</v>
       </c>
       <c r="E74" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="G74" s="0" t="s">
-        <v>316</v>
+        <v>340</v>
       </c>
       <c r="H74" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I74" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="75">
@@ -3370,22 +3445,22 @@
         <v>176</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E75" s="0" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F75" s="0" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="G75" s="0" t="s">
-        <v>317</v>
+        <v>341</v>
       </c>
       <c r="H75" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I75" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="76">
@@ -3402,19 +3477,19 @@
         <v>113</v>
       </c>
       <c r="E76" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F76" s="0" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
       <c r="G76" s="0" t="s">
-        <v>318</v>
+        <v>342</v>
       </c>
       <c r="H76" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="77">
@@ -3428,22 +3503,22 @@
         <v>178</v>
       </c>
       <c r="D77" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="E77" s="0" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="G77" s="0" t="s">
-        <v>319</v>
+        <v>343</v>
       </c>
       <c r="H77" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I77" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="78">
@@ -3460,19 +3535,19 @@
         <v>113</v>
       </c>
       <c r="E78" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
       <c r="G78" s="0" t="s">
-        <v>320</v>
+        <v>344</v>
       </c>
       <c r="H78" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I78" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="79">
@@ -3486,22 +3561,22 @@
         <v>180</v>
       </c>
       <c r="D79" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E79" s="0" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F79" s="0" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
       <c r="G79" s="0" t="s">
-        <v>321</v>
+        <v>345</v>
       </c>
       <c r="H79" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I79" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="80">
@@ -3518,19 +3593,19 @@
         <v>113</v>
       </c>
       <c r="E80" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="G80" s="0" t="s">
-        <v>322</v>
+        <v>346</v>
       </c>
       <c r="H80" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I80" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="81">
@@ -3544,22 +3619,22 @@
         <v>182</v>
       </c>
       <c r="D81" s="0" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E81" s="0" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F81" s="0" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="G81" s="0" t="s">
-        <v>307</v>
+        <v>347</v>
       </c>
       <c r="H81" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I81" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="82">
@@ -3576,19 +3651,19 @@
         <v>113</v>
       </c>
       <c r="E82" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="G82" s="0" t="s">
-        <v>323</v>
+        <v>348</v>
       </c>
       <c r="H82" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I82" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="83">
@@ -3605,19 +3680,19 @@
         <v>141</v>
       </c>
       <c r="E83" s="0" t="s">
-        <v>224</v>
+        <v>249</v>
       </c>
       <c r="F83" s="0" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="G83" s="0" t="s">
-        <v>324</v>
+        <v>349</v>
       </c>
       <c r="H83" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I83" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="84">
@@ -3631,22 +3706,22 @@
         <v>185</v>
       </c>
       <c r="D84" s="0" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E84" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F84" s="0" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="G84" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H84" s="0" t="s">
         <v>113</v>
       </c>
       <c r="I84" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sizing/reporting: update aero comparison reports for L2's new LEF term
aerodynamics_brandt_comparison.m's "CLmax takeoff/landing (L2 flap)" rows
and note text claimed "no slat at L2" -- now false. Relabel to "L2
flap+slat", update the notes to point at the fidelity-gap closure, and
regenerate the committed JSON/Markdown outputs from a live run.

fidelity_comparison.m's high-lift-device legend described L2 as "flap
only" and L3 as the one that "adds the LE slat" -- rewritten to describe
both levels as sharing identical flaperon/LEF formulas via the injected
ControlSurfaceSizer, with only the gear-drag buildup remaining L3-exclusive.
Regenerated the committed JSON/Excel outputs from a live run.
</commit_message>
<xml_diff>
--- a/air_vehicle_design/sizing/examples/F16A/fidelity_comparison.xlsx
+++ b/air_vehicle_design/sizing/examples/F16A/fidelity_comparison.xlsx
@@ -1,7 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fileVersion appName="libxl" rupBuild="4.6.0"/>
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -14,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="756" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="756" uniqueCount="380">
   <si>
     <t>Row</t>
   </si>
@@ -814,34 +813,34 @@
     <t>2.9179</t>
   </si>
   <si>
-    <t>0.0344</t>
-  </si>
-  <si>
-    <t>0.0488</t>
-  </si>
-  <si>
-    <t>0.0515</t>
-  </si>
-  <si>
-    <t>0.0659</t>
-  </si>
-  <si>
-    <t>0.3291</t>
-  </si>
-  <si>
-    <t>0.4387</t>
-  </si>
-  <si>
-    <t>1.2431</t>
-  </si>
-  <si>
-    <t>1.3528</t>
-  </si>
-  <si>
-    <t>0.0257</t>
-  </si>
-  <si>
-    <t>0.0456</t>
+    <t>0.0418</t>
+  </si>
+  <si>
+    <t>0.0485</t>
+  </si>
+  <si>
+    <t>0.0589</t>
+  </si>
+  <si>
+    <t>0.0656</t>
+  </si>
+  <si>
+    <t>0.1788</t>
+  </si>
+  <si>
+    <t>0.2384</t>
+  </si>
+  <si>
+    <t>1.0929</t>
+  </si>
+  <si>
+    <t>1.1525</t>
+  </si>
+  <si>
+    <t>0.0057</t>
+  </si>
+  <si>
+    <t>0.0101</t>
   </si>
   <si>
     <t>0.0446</t>
@@ -958,22 +957,22 @@
     <t>-6.2%</t>
   </si>
   <si>
-    <t>-0.9%</t>
-  </si>
-  <si>
-    <t>+6.3%</t>
-  </si>
-  <si>
-    <t>+12.0%</t>
-  </si>
-  <si>
-    <t>-1.4%</t>
-  </si>
-  <si>
-    <t>-2.7%</t>
-  </si>
-  <si>
-    <t>-5.3%</t>
+    <t>+13.2%</t>
+  </si>
+  <si>
+    <t>+5.8%</t>
+  </si>
+  <si>
+    <t>-39.1%</t>
+  </si>
+  <si>
+    <t>-46.4%</t>
+  </si>
+  <si>
+    <t>-14.5%</t>
+  </si>
+  <si>
+    <t>-19.4%</t>
   </si>
   <si>
     <t>-3.3%</t>
@@ -1018,10 +1017,10 @@
     <t>L3</t>
   </si>
   <si>
-    <t>15795</t>
-  </si>
-  <si>
-    <t>0.5034</t>
+    <t>15790</t>
+  </si>
+  <si>
+    <t>0.5032</t>
   </si>
   <si>
     <t>2397</t>
@@ -1042,7 +1041,7 @@
     <t>3382</t>
   </si>
   <si>
-    <t>4578</t>
+    <t>4573</t>
   </si>
   <si>
     <t>1488.3</t>
@@ -1066,22 +1065,10 @@
     <t>0.0351</t>
   </si>
   <si>
-    <t>0.0486</t>
-  </si>
-  <si>
-    <t>0.0648</t>
-  </si>
-  <si>
-    <t>0.3537</t>
-  </si>
-  <si>
-    <t>0.4716</t>
-  </si>
-  <si>
-    <t>1.2677</t>
-  </si>
-  <si>
-    <t>1.3856</t>
+    <t>0.0333</t>
+  </si>
+  <si>
+    <t>0.0495</t>
   </si>
   <si>
     <t>0.0388</t>
@@ -1102,7 +1089,7 @@
     <t>L3_err</t>
   </si>
   <si>
-    <t>-20.9%</t>
+    <t>-21.0%</t>
   </si>
   <si>
     <t>+34.2%</t>
@@ -1120,7 +1107,7 @@
     <t>-40.1%</t>
   </si>
   <si>
-    <t>-32.9%</t>
+    <t>-33.0%</t>
   </si>
   <si>
     <t>+8.5%</t>
@@ -1144,22 +1131,10 @@
     <t>-3.9%</t>
   </si>
   <si>
-    <t>+24.7%</t>
-  </si>
-  <si>
-    <t>+4.6%</t>
-  </si>
-  <si>
-    <t>+20.4%</t>
-  </si>
-  <si>
-    <t>+6.0%</t>
-  </si>
-  <si>
-    <t>-0.8%</t>
-  </si>
-  <si>
-    <t>-3.0%</t>
+    <t>-4.8%</t>
+  </si>
+  <si>
+    <t>-20.1%</t>
   </si>
   <si>
     <t>-15.8%</t>
@@ -1263,7 +1238,7 @@
         <v>333</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2">
@@ -1321,7 +1296,7 @@
         <v>334</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4">
@@ -1350,7 +1325,7 @@
         <v>335</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
     </row>
     <row r="5">
@@ -1379,7 +1354,7 @@
         <v>336</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="6">
@@ -1408,7 +1383,7 @@
         <v>337</v>
       </c>
       <c r="I6" s="0" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7">
@@ -1437,7 +1412,7 @@
         <v>338</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
     <row r="8">
@@ -1495,7 +1470,7 @@
         <v>340</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
     </row>
     <row r="10">
@@ -1524,7 +1499,7 @@
         <v>341</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
     </row>
     <row r="11">
@@ -1553,7 +1528,7 @@
         <v>342</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
     </row>
     <row r="12">
@@ -1611,7 +1586,7 @@
         <v>343</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="14">
@@ -1698,7 +1673,7 @@
         <v>344</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
     </row>
     <row r="17">
@@ -1756,7 +1731,7 @@
         <v>345</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
     </row>
     <row r="19">
@@ -1843,7 +1818,7 @@
         <v>258</v>
       </c>
       <c r="I21" s="0" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
     </row>
     <row r="22">
@@ -1872,7 +1847,7 @@
         <v>346</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
     </row>
     <row r="23">
@@ -1901,7 +1876,7 @@
         <v>347</v>
       </c>
       <c r="I23" s="0" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
     </row>
     <row r="24">
@@ -1930,7 +1905,7 @@
         <v>348</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
     </row>
     <row r="25">
@@ -2394,7 +2369,7 @@
         <v>351</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
     </row>
     <row r="41">
@@ -2423,7 +2398,7 @@
         <v>351</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="42">
@@ -2449,10 +2424,10 @@
         <v>316</v>
       </c>
       <c r="H42" s="0" t="s">
-        <v>352</v>
+        <v>270</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>378</v>
+        <v>316</v>
       </c>
     </row>
     <row r="43">
@@ -2478,10 +2453,10 @@
         <v>317</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>353</v>
+        <v>271</v>
       </c>
       <c r="I43" s="0" t="s">
-        <v>379</v>
+        <v>317</v>
       </c>
     </row>
     <row r="44">
@@ -2507,10 +2482,10 @@
         <v>318</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>354</v>
+        <v>272</v>
       </c>
       <c r="I44" s="0" t="s">
-        <v>380</v>
+        <v>318</v>
       </c>
     </row>
     <row r="45">
@@ -2536,10 +2511,10 @@
         <v>319</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>355</v>
+        <v>273</v>
       </c>
       <c r="I45" s="0" t="s">
-        <v>381</v>
+        <v>319</v>
       </c>
     </row>
     <row r="46">
@@ -2594,7 +2569,7 @@
         <v>212</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>103</v>
+        <v>275</v>
       </c>
       <c r="I47" s="0" t="s">
         <v>212</v>
@@ -2652,10 +2627,10 @@
         <v>320</v>
       </c>
       <c r="H49" s="0" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="I49" s="0" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
     </row>
     <row r="50">
@@ -2739,10 +2714,10 @@
         <v>219</v>
       </c>
       <c r="H52" s="0" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
     </row>
     <row r="53">
@@ -2826,10 +2801,10 @@
         <v>219</v>
       </c>
       <c r="H55" s="0" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="I55" s="0" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
     </row>
     <row r="56">
@@ -2913,10 +2888,10 @@
         <v>322</v>
       </c>
       <c r="H58" s="0" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="I58" s="0" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
     </row>
     <row r="59">
@@ -3000,10 +2975,10 @@
         <v>219</v>
       </c>
       <c r="H61" s="0" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="I61" s="0" t="s">
-        <v>386</v>
+        <v>378</v>
       </c>
     </row>
     <row r="62">
@@ -3087,10 +3062,10 @@
         <v>323</v>
       </c>
       <c r="H64" s="0" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="I64" s="0" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
     </row>
     <row r="65">
@@ -3177,7 +3152,7 @@
         <v>346</v>
       </c>
       <c r="I67" s="0" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
     </row>
     <row r="68">

</xml_diff>